<commit_message>
[CB] Removed .2f float point format restriction when merging bills metadata
</commit_message>
<xml_diff>
--- a/congressional_bills/01_bills/bills_codebook.xlsx
+++ b/congressional_bills/01_bills/bills_codebook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/haya1/Documents/LanguageModel_Labels/congressional_bills/01_bills/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{232DE661-FF70-F54D-9110-E9265BE285D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E7CDA0A-C9D3-134E-9ED3-979EA663C885}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="780" yWindow="1180" windowWidth="27640" windowHeight="15760" xr2:uid="{780D6C32-B720-8E44-8C6F-66FB360933E5}"/>
   </bookViews>
@@ -182,9 +182,6 @@
     <t>Title bill with minor corrections</t>
   </si>
   <si>
-    <t>Party code of the bill sponser at the time of introduction using ICPSR coding scheme (100: Democrat; 112: Conservative; 200: Republican, 328: Independent)</t>
-  </si>
-  <si>
     <t>Sponser's first dimension DW-NOMINATE score (i.e., sponser's score on liberal-conservative spectrum on economic matters). Missing values are included as Blank/NaNs</t>
   </si>
   <si>
@@ -287,6 +284,9 @@
   <si>
     <t>Variable codes in CBP follows the coding scheme of ICPSR. The original link (http://www.icpsr.umich.edu/cgi-bin/file?comp=none&amp;study=3371&amp;ds=2&amp;file_id=965434&amp;path=ICPSR) doesn't work. Maybe they mean (https://www.icpsr.umich.edu/web/ICPSR/studies/3371)? TODO: correct this</t>
   </si>
+  <si>
+    <t>Party code of the bill sponser at the time of introduction using ICPSR coding scheme (100: Democrat; 200: Republican, 328: Independent)</t>
+  </si>
 </sst>
 </file>
 
@@ -362,7 +362,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -373,13 +373,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -391,7 +385,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -739,250 +733,250 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A1" s="7" t="s">
-        <v>66</v>
+      <c r="A1" s="5" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B2" s="1"/>
       <c r="D2"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B3" s="1"/>
       <c r="D3"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B4" s="1"/>
       <c r="D4"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B5" s="1"/>
       <c r="D5"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8" s="7" t="s">
-        <v>59</v>
+      <c r="A8" s="5" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B9" s="9" t="s">
-        <v>60</v>
+      <c r="B9" s="7" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="8" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="68" x14ac:dyDescent="0.2">
+      <c r="A11" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B12" s="2"/>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A13" s="2"/>
+    </row>
+    <row r="14" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A14" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="C14" s="5" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="68" x14ac:dyDescent="0.2">
-      <c r="A11" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="B11" s="10" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B12" s="2"/>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A13" s="2"/>
-    </row>
-    <row r="14" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A14" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="B14" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="C14" s="7" t="s">
-        <v>63</v>
-      </c>
-    </row>
     <row r="15" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A15" s="4" t="s">
+      <c r="A15" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C15" s="1" t="s">
         <v>36</v>
       </c>
       <c r="D15"/>
     </row>
     <row r="16" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A16" s="4" t="s">
+      <c r="A16" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="B16" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C16" s="1" t="s">
         <v>36</v>
       </c>
       <c r="D16"/>
     </row>
     <row r="17" spans="1:7" ht="68" x14ac:dyDescent="0.2">
-      <c r="A17" s="4" t="s">
+      <c r="A17" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B17" s="6" t="s">
-        <v>57</v>
+      <c r="B17" s="4" t="s">
+        <v>56</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="C17" s="1" t="s">
         <v>36</v>
       </c>
       <c r="D17"/>
       <c r="E17" s="2"/>
     </row>
     <row r="18" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A18" s="4" t="s">
+      <c r="A18" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B18" s="6" t="s">
-        <v>58</v>
+      <c r="B18" s="4" t="s">
+        <v>57</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="C18" s="1" t="s">
         <v>36</v>
       </c>
       <c r="D18"/>
       <c r="E18" s="2"/>
     </row>
     <row r="19" spans="1:7" ht="34" x14ac:dyDescent="0.2">
-      <c r="A19" s="4" t="s">
+      <c r="A19" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B19" s="6" t="s">
-        <v>48</v>
+      <c r="B19" s="4" t="s">
+        <v>69</v>
       </c>
-      <c r="C19" s="4" t="s">
+      <c r="C19" s="1" t="s">
         <v>36</v>
       </c>
       <c r="D19"/>
       <c r="E19" s="2"/>
     </row>
     <row r="20" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A20" s="4" t="s">
+      <c r="A20" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B20" s="6" t="s">
+      <c r="B20" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="C20" s="4" t="s">
+      <c r="C20" s="1" t="s">
         <v>36</v>
       </c>
       <c r="D20"/>
       <c r="E20" s="2"/>
     </row>
     <row r="21" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A21" s="4" t="s">
+      <c r="A21" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B21" s="6" t="s">
+      <c r="B21" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="C21" s="4" t="s">
+      <c r="C21" s="1" t="s">
         <v>36</v>
       </c>
       <c r="D21"/>
       <c r="E21" s="2"/>
     </row>
     <row r="22" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A22" s="4" t="s">
+      <c r="A22" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B22" s="6" t="s">
+      <c r="B22" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="C22" s="4" t="s">
+      <c r="C22" s="1" t="s">
         <v>36</v>
       </c>
       <c r="D22"/>
       <c r="E22" s="2"/>
     </row>
     <row r="23" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A23" s="4" t="s">
-        <v>53</v>
+      <c r="A23" s="1" t="s">
+        <v>52</v>
       </c>
-      <c r="B23" s="6" t="s">
-        <v>56</v>
+      <c r="B23" s="4" t="s">
+        <v>55</v>
       </c>
-      <c r="C23" s="4" t="s">
+      <c r="C23" s="1" t="s">
         <v>35</v>
       </c>
       <c r="D23"/>
       <c r="E23" s="2"/>
     </row>
     <row r="24" spans="1:7" ht="34" x14ac:dyDescent="0.2">
-      <c r="A24" s="4" t="s">
+      <c r="A24" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B24" s="6" t="s">
-        <v>49</v>
+      <c r="B24" s="4" t="s">
+        <v>48</v>
       </c>
-      <c r="C24" s="4" t="s">
+      <c r="C24" s="1" t="s">
         <v>35</v>
       </c>
       <c r="D24"/>
       <c r="E24" s="2"/>
     </row>
     <row r="25" spans="1:7" ht="34" x14ac:dyDescent="0.2">
-      <c r="A25" s="4" t="s">
+      <c r="A25" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B25" s="5" t="s">
-        <v>50</v>
+      <c r="B25" s="3" t="s">
+        <v>49</v>
       </c>
-      <c r="C25" s="4" t="s">
+      <c r="C25" s="1" t="s">
         <v>35</v>
       </c>
       <c r="D25"/>
     </row>
     <row r="26" spans="1:7" ht="34" x14ac:dyDescent="0.2">
-      <c r="A26" s="4" t="s">
+      <c r="A26" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B26" s="6" t="s">
-        <v>64</v>
+      <c r="B26" s="4" t="s">
+        <v>63</v>
       </c>
-      <c r="C26" s="4" t="s">
+      <c r="C26" s="1" t="s">
         <v>36</v>
       </c>
       <c r="D26"/>
       <c r="G26" s="2"/>
     </row>
     <row r="27" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A27" s="4" t="s">
+      <c r="A27" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B27" s="6" t="s">
+      <c r="B27" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="C27" s="4" t="s">
+      <c r="C27" s="1" t="s">
         <v>35</v>
       </c>
       <c r="D27"/>
@@ -990,78 +984,78 @@
       <c r="G27" s="2"/>
     </row>
     <row r="28" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A28" s="4" t="s">
+      <c r="A28" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B28" s="6" t="s">
+      <c r="B28" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="C28" s="4" t="s">
+      <c r="C28" s="1" t="s">
         <v>35</v>
       </c>
       <c r="D28"/>
       <c r="G28" s="2"/>
     </row>
     <row r="29" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A29" s="4" t="s">
+      <c r="A29" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B29" s="6" t="s">
+      <c r="B29" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C29" s="4" t="s">
+      <c r="C29" s="1" t="s">
         <v>35</v>
       </c>
       <c r="D29"/>
       <c r="G29" s="2"/>
     </row>
     <row r="30" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A30" s="4" t="s">
+      <c r="A30" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B30" s="6" t="s">
-        <v>51</v>
+      <c r="B30" s="4" t="s">
+        <v>50</v>
       </c>
-      <c r="C30" s="4" t="s">
+      <c r="C30" s="1" t="s">
         <v>35</v>
       </c>
       <c r="D30"/>
       <c r="G30" s="2"/>
     </row>
     <row r="31" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A31" s="4" t="s">
+      <c r="A31" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B31" s="6" t="s">
+      <c r="B31" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C31" s="4" t="s">
+      <c r="C31" s="1" t="s">
         <v>35</v>
       </c>
       <c r="D31"/>
       <c r="G31" s="2"/>
     </row>
     <row r="32" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A32" s="4" t="s">
+      <c r="A32" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B32" s="6" t="s">
+      <c r="B32" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C32" s="4" t="s">
+      <c r="C32" s="1" t="s">
         <v>35</v>
       </c>
       <c r="D32"/>
       <c r="G32" s="2"/>
     </row>
     <row r="33" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A33" s="4" t="s">
+      <c r="A33" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B33" s="6" t="s">
+      <c r="B33" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="C33" s="4" t="s">
+      <c r="C33" s="1" t="s">
         <v>35</v>
       </c>
       <c r="D33"/>
@@ -1069,26 +1063,26 @@
       <c r="G33" s="2"/>
     </row>
     <row r="34" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A34" s="4" t="s">
+      <c r="A34" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B34" s="6" t="s">
+      <c r="B34" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="C34" s="4" t="s">
+      <c r="C34" s="1" t="s">
         <v>35</v>
       </c>
       <c r="D34"/>
       <c r="G34" s="2"/>
     </row>
     <row r="35" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A35" s="4" t="s">
+      <c r="A35" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B35" s="6" t="s">
+      <c r="B35" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C35" s="4" t="s">
+      <c r="C35" s="1" t="s">
         <v>35</v>
       </c>
       <c r="D35"/>
@@ -1096,26 +1090,26 @@
       <c r="G35" s="2"/>
     </row>
     <row r="36" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A36" s="4" t="s">
+      <c r="A36" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B36" s="6" t="s">
+      <c r="B36" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="C36" s="4" t="s">
+      <c r="C36" s="1" t="s">
         <v>35</v>
       </c>
       <c r="D36"/>
       <c r="G36" s="2"/>
     </row>
     <row r="37" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A37" s="4" t="s">
+      <c r="A37" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B37" s="6" t="s">
+      <c r="B37" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="C37" s="4" t="s">
+      <c r="C37" s="1" t="s">
         <v>35</v>
       </c>
       <c r="D37"/>
@@ -1123,52 +1117,52 @@
       <c r="G37" s="2"/>
     </row>
     <row r="38" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A38" s="4" t="s">
+      <c r="A38" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B38" s="6" t="s">
+      <c r="B38" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="C38" s="4" t="s">
+      <c r="C38" s="1" t="s">
         <v>35</v>
       </c>
       <c r="D38"/>
       <c r="G38" s="2"/>
     </row>
     <row r="39" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A39" s="4" t="s">
+      <c r="A39" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B39" s="6" t="s">
-        <v>52</v>
+      <c r="B39" s="4" t="s">
+        <v>51</v>
       </c>
-      <c r="C39" s="4" t="s">
+      <c r="C39" s="1" t="s">
         <v>35</v>
       </c>
       <c r="D39"/>
       <c r="G39" s="2"/>
     </row>
     <row r="40" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A40" s="4" t="s">
+      <c r="A40" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B40" s="6" t="s">
+      <c r="B40" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="C40" s="4" t="s">
+      <c r="C40" s="1" t="s">
         <v>35</v>
       </c>
       <c r="D40"/>
       <c r="G40" s="2"/>
     </row>
     <row r="41" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A41" s="4" t="s">
+      <c r="A41" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B41" s="6" t="s">
+      <c r="B41" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="C41" s="4" t="s">
+      <c r="C41" s="1" t="s">
         <v>35</v>
       </c>
       <c r="D41"/>

</xml_diff>

<commit_message>
[CB] Added codes for Party and Congress variables
</commit_message>
<xml_diff>
--- a/congressional_bills/01_bills/bills_codebook.xlsx
+++ b/congressional_bills/01_bills/bills_codebook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/haya1/Documents/LanguageModel_Labels/congressional_bills/01_bills/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E7CDA0A-C9D3-134E-9ED3-979EA663C885}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{481148F8-5D9E-3D40-B8D1-9EC1B3352586}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="780" yWindow="1180" windowWidth="27640" windowHeight="15760" xr2:uid="{780D6C32-B720-8E44-8C6F-66FB360933E5}"/>
   </bookViews>
@@ -125,9 +125,6 @@
     <t>State</t>
   </si>
   <si>
-    <t>Numeric code of home state (ICPSR)</t>
-  </si>
-  <si>
     <t>Year</t>
   </si>
   <si>
@@ -159,9 +156,6 @@
   </si>
   <si>
     <t>1: Vetoed by the President; 0: Otherwise</t>
-  </si>
-  <si>
-    <t>Postal code of home state (e.g. WA)</t>
   </si>
   <si>
     <t>Variable Name</t>
@@ -285,7 +279,13 @@
     <t>Variable codes in CBP follows the coding scheme of ICPSR. The original link (http://www.icpsr.umich.edu/cgi-bin/file?comp=none&amp;study=3371&amp;ds=2&amp;file_id=965434&amp;path=ICPSR) doesn't work. Maybe they mean (https://www.icpsr.umich.edu/web/ICPSR/studies/3371)? TODO: correct this</t>
   </si>
   <si>
-    <t>Party code of the bill sponser at the time of introduction using ICPSR coding scheme (100: Democrat; 200: Republican, 328: Independent)</t>
+    <t>Postal code of home state, e.g. AK, AL, AR, …</t>
+  </si>
+  <si>
+    <t>Numeric code of home state using ICPSR coding, e.g., 0: Not categorized (AS, GU, MP, PR, VI); 1: CT, 2: ME, …</t>
+  </si>
+  <si>
+    <t>Party code of the bill sponser at the time of introduction using ICPSR coding scheme (100: Democrat; 112: Conservative; 200: Republican, 328: Independent)</t>
   </si>
 </sst>
 </file>
@@ -734,71 +734,71 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="5" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B2" s="1"/>
       <c r="D2"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B3" s="1"/>
       <c r="D3"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B4" s="1"/>
       <c r="D4"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B5" s="1"/>
       <c r="D5"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8" s="5" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="A9" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="A10" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="68" x14ac:dyDescent="0.2">
+      <c r="A11" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B11" s="8" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8" s="5" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="34" x14ac:dyDescent="0.2">
-      <c r="A9" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="B9" s="7" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="34" x14ac:dyDescent="0.2">
-      <c r="A10" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="B10" s="8" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="68" x14ac:dyDescent="0.2">
-      <c r="A11" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="B11" s="8" t="s">
-        <v>68</v>
-      </c>
-    </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B12" s="2"/>
     </row>
@@ -807,13 +807,13 @@
     </row>
     <row r="14" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A14" s="5" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="17" x14ac:dyDescent="0.2">
@@ -821,22 +821,22 @@
         <v>0</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D15"/>
     </row>
     <row r="16" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D16"/>
     </row>
@@ -845,23 +845,23 @@
         <v>7</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D17"/>
       <c r="E17" s="2"/>
     </row>
     <row r="18" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D18"/>
       <c r="E18" s="2"/>
@@ -874,7 +874,7 @@
         <v>69</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D19"/>
       <c r="E19" s="2"/>
@@ -884,10 +884,10 @@
         <v>11</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D20"/>
       <c r="E20" s="2"/>
@@ -897,36 +897,36 @@
         <v>12</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D21"/>
       <c r="E21" s="2"/>
     </row>
     <row r="22" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D22"/>
       <c r="E22" s="2"/>
     </row>
     <row r="23" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D23"/>
       <c r="E23" s="2"/>
@@ -936,23 +936,23 @@
         <v>22</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D24"/>
       <c r="E24" s="2"/>
     </row>
     <row r="25" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D25"/>
     </row>
@@ -961,10 +961,10 @@
         <v>4</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D26"/>
       <c r="G26" s="2"/>
@@ -977,7 +977,7 @@
         <v>2</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D27"/>
       <c r="E27" s="2"/>
@@ -988,10 +988,10 @@
         <v>3</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D28"/>
       <c r="G28" s="2"/>
@@ -1004,7 +1004,7 @@
         <v>6</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D29"/>
       <c r="G29" s="2"/>
@@ -1014,10 +1014,10 @@
         <v>8</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D30"/>
       <c r="G30" s="2"/>
@@ -1030,7 +1030,7 @@
         <v>10</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D31"/>
       <c r="G31" s="2"/>
@@ -1043,7 +1043,7 @@
         <v>14</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D32"/>
       <c r="G32" s="2"/>
@@ -1053,10 +1053,10 @@
         <v>15</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D33"/>
       <c r="E33" s="2"/>
@@ -1067,10 +1067,10 @@
         <v>16</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D34"/>
       <c r="G34" s="2"/>
@@ -1080,10 +1080,10 @@
         <v>17</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D35"/>
       <c r="E35" s="2"/>
@@ -1097,7 +1097,7 @@
         <v>19</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D36"/>
       <c r="G36" s="2"/>
@@ -1110,7 +1110,7 @@
         <v>21</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D37"/>
       <c r="E37" s="2"/>
@@ -1124,7 +1124,7 @@
         <v>24</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D38"/>
       <c r="G38" s="2"/>
@@ -1134,10 +1134,10 @@
         <v>25</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D39"/>
       <c r="G39" s="2"/>
@@ -1147,23 +1147,23 @@
         <v>27</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>41</v>
+        <v>67</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D40"/>
       <c r="G40" s="2"/>
     </row>
-    <row r="41" spans="1:7" ht="17" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
         <v>28</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>29</v>
+        <v>68</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D41"/>
       <c r="E41" s="2"/>

</xml_diff>